<commit_message>
Update all validation sheets with implemented fixes reflected
</commit_message>
<xml_diff>
--- a/step1-validation-test.xlsx
+++ b/step1-validation-test.xlsx
@@ -447,7 +447,7 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -525,7 +525,7 @@
           <t>「(例) YAMADA」が表示</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
@@ -557,7 +557,7 @@
           <t>エラー表示/進めない</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
@@ -589,7 +589,7 @@
           <t>45文字で止まる</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -621,7 +621,7 @@
           <t>数字除去「YAMADA」</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
@@ -653,7 +653,7 @@
           <t>除去される</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
@@ -685,7 +685,7 @@
           <t>記号除去「YAMADA」</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
@@ -717,7 +717,7 @@
           <t>「YAMADA」に変換</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
@@ -749,7 +749,7 @@
           <t>「YAMADA TANAKA」に</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
@@ -781,7 +781,7 @@
           <t>「YAMADA」に</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
@@ -813,7 +813,7 @@
           <t>確認アラート表示</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
@@ -845,7 +845,7 @@
           <t>「半角英字で入力してください」表示</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -877,7 +877,7 @@
           <t>ボタン非アクティブ</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
@@ -909,7 +909,7 @@
           <t>「(例) TARO」表示</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
@@ -941,7 +941,7 @@
           <t>パスポート記載通りの注記</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
@@ -973,7 +973,7 @@
           <t>全て姓と同様に動作</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1005,7 +1005,7 @@
           <t>「別名はありません」選択</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1037,7 +1037,7 @@
           <t>姓名(別名)表示</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1069,7 +1069,7 @@
           <t>入力欄非表示</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1101,7 +1101,7 @@
           <t>同一動作</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1133,7 +1133,7 @@
           <t>同一動作</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1165,7 +1165,7 @@
           <t>どちらも未選択</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1197,7 +1197,7 @@
           <t>選択状態</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1229,7 +1229,7 @@
           <t>選択状態</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
       <c r="H24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1261,7 +1261,7 @@
           <t>「Unspecified」追加</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1293,7 +1293,7 @@
           <t>Year年Month月Day日</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1325,7 +1325,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1357,7 +1357,7 @@
           <t>エラー表示+月日リセット</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1389,7 +1389,7 @@
           <t>JAPAN(JPN)選択</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1421,7 +1421,7 @@
           <t>SOUTH KOREA絞り込み</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
       <c r="H30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1453,7 +1453,7 @@
           <t>ボタン非アクティブ</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1485,7 +1485,7 @@
           <t>フィールド表示</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1517,7 +1517,7 @@
           <t>フィールド非表示</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1549,7 +1549,7 @@
           <t>全て表示</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
       <c r="H34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1581,7 +1581,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
       <c r="H35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1613,7 +1613,7 @@
           <t>除去</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
       <c r="H36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1645,7 +1645,7 @@
           <t>変換される</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1677,7 +1677,7 @@
           <t>除去</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
       <c r="H38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1709,7 +1709,7 @@
           <t>必須フィールド表示</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1741,7 +1741,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1773,7 +1773,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1805,7 +1805,7 @@
           <t>10文字で止まる</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1837,7 +1837,7 @@
           <t>yamada_taro@example.co.jp表示</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
       <c r="H43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1869,7 +1869,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
       <c r="H44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1901,7 +1901,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1933,7 +1933,7 @@
           <t>半角に変換</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
       <c r="H46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1965,7 +1965,7 @@
           <t>trimされる</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
@@ -1997,7 +1997,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr"/>
       <c r="H48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2029,7 +2029,7 @@
           <t>「一致しません」表示</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2061,7 +2061,7 @@
           <t>JAPAN (+81)</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr"/>
       <c r="H50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2093,7 +2093,7 @@
           <t>英字除去+20桁制限</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2125,7 +2125,7 @@
           <t>半角に変換</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr"/>
       <c r="H52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2157,7 +2157,7 @@
           <t>09012345678に</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
       <c r="H53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2189,7 +2189,7 @@
           <t>自宅/勤務先/携帯/その他</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr"/>
       <c r="H54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
@@ -2221,7 +2221,7 @@
           <t>ボタン非アクティブ</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
       <c r="H55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
@@ -2253,7 +2253,7 @@
           <t>除去</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr"/>
       <c r="H56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2285,7 +2285,7 @@
           <t>都道府県/市区町村自動入力</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2317,7 +2317,7 @@
           <t>アラート表示</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr"/>
+      <c r="G58" s="4" t="inlineStr"/>
       <c r="H58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
@@ -2349,7 +2349,7 @@
           <t>郵便局サイトに遷移</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2381,7 +2381,7 @@
           <t>JAPAN(JPN)選択</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="G60" s="4" t="inlineStr"/>
       <c r="H60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
@@ -2413,7 +2413,7 @@
           <t>数字除去TOKYO</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
       <c r="H61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
@@ -2445,7 +2445,7 @@
           <t>TOKYO</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr"/>
       <c r="H62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
@@ -2477,7 +2477,7 @@
           <t>許可</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr"/>
       <c r="H63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
@@ -2509,7 +2509,7 @@
           <t>許可</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr"/>
+      <c r="G64" s="4" t="inlineStr"/>
       <c r="H64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
@@ -2541,7 +2541,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr"/>
       <c r="H65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
@@ -2573,7 +2573,7 @@
           <t>101に</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr"/>
       <c r="H66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
@@ -2605,7 +2605,7 @@
           <t>ファイル名が表示される</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
       <c r="H67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
@@ -2637,7 +2637,7 @@
           <t>エラー「サイズが上限の10MBを超えています」</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="G68" s="4" t="inlineStr"/>
       <c r="H68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
@@ -2669,7 +2669,7 @@
           <t>ファイル選択ダイアログで制限</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
       <c r="H69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
@@ -2701,7 +2701,7 @@
           <t>ファイル名が表示</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr"/>
+      <c r="G70" s="4" t="inlineStr"/>
       <c r="H70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
@@ -2733,7 +2733,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr"/>
       <c r="H71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
@@ -2765,7 +2765,7 @@
           <t>「jpeg,pngファイルのみ」エラー</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr"/>
+      <c r="G72" s="4" t="inlineStr"/>
       <c r="H72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2797,7 +2797,7 @@
           <t>パスポート顔写真使用不可の赤字注記</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr"/>
       <c r="H73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
@@ -2829,7 +2829,7 @@
           <t>(例) TH1234567</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr"/>
+      <c r="G74" s="4" t="inlineStr"/>
       <c r="H74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
@@ -2861,7 +2861,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
       <c r="H75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
@@ -2893,7 +2893,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr"/>
+      <c r="G76" s="4" t="inlineStr"/>
       <c r="H76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
@@ -2925,7 +2925,7 @@
           <t>TH1234567に変換</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr"/>
       <c r="H77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
@@ -2957,7 +2957,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr"/>
+      <c r="G78" s="4" t="inlineStr"/>
       <c r="H78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
@@ -2989,7 +2989,7 @@
           <t>O(オー)と0(ゼロ)の混同注意</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr"/>
       <c r="H79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3021,7 +3021,7 @@
           <t>Day日/Month月/Year年</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr"/>
+      <c r="G80" s="4" t="inlineStr"/>
       <c r="H80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
@@ -3053,7 +3053,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr"/>
       <c r="H81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
@@ -3085,7 +3085,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr"/>
+      <c r="G82" s="4" t="inlineStr"/>
       <c r="H82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
@@ -3117,7 +3117,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr"/>
       <c r="H83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
@@ -3149,7 +3149,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr"/>
       <c r="H84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
@@ -3181,7 +3181,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr"/>
       <c r="H85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
@@ -3213,7 +3213,7 @@
           <t>正常/不一致で訂正旅券注記</t>
         </is>
       </c>
-      <c r="G86" s="2" t="inlineStr"/>
+      <c r="G86" s="4" t="inlineStr"/>
       <c r="H86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
@@ -3245,7 +3245,7 @@
           <t>正常/不一致で訂正旅券注記</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr"/>
       <c r="H87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
@@ -3277,7 +3277,7 @@
           <t>JAPAN(JPN)選択</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr"/>
       <c r="H88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
@@ -3309,7 +3309,7 @@
           <t>※通常は国籍と同じ</t>
         </is>
       </c>
-      <c r="G89" s="2" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr"/>
       <c r="H89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
@@ -3341,7 +3341,7 @@
           <t>JAPAN(JPN)選択</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr"/>
+      <c r="G90" s="4" t="inlineStr"/>
       <c r="H90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
@@ -3373,7 +3373,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr"/>
       <c r="H91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
@@ -3405,7 +3405,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr"/>
       <c r="H92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
@@ -3437,7 +3437,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr"/>
+      <c r="G93" s="4" t="inlineStr"/>
       <c r="H93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
@@ -3469,7 +3469,7 @@
           <t>「いいえ」選択</t>
         </is>
       </c>
-      <c r="G94" s="2" t="inlineStr"/>
+      <c r="G94" s="4" t="inlineStr"/>
       <c r="H94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
@@ -3501,7 +3501,7 @@
           <t>発給国/種類/ID/期限の入力欄表示</t>
         </is>
       </c>
-      <c r="G95" s="2" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr"/>
       <c r="H95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
@@ -3533,7 +3533,7 @@
           <t>入力欄非表示</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr"/>
       <c r="H96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
@@ -3565,7 +3565,7 @@
           <t>正常に選択</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr"/>
+      <c r="G97" s="4" t="inlineStr"/>
       <c r="H97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
@@ -3597,7 +3597,7 @@
           <t>パスポート/国家身分証明書</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr"/>
+      <c r="G98" s="4" t="inlineStr"/>
       <c r="H98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
@@ -3629,7 +3629,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr"/>
       <c r="H99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
@@ -3661,7 +3661,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr"/>
+      <c r="G100" s="4" t="inlineStr"/>
       <c r="H100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
@@ -3693,7 +3693,7 @@
           <t>UNKNOWN含む選択肢</t>
         </is>
       </c>
-      <c r="G101" s="2" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr"/>
       <c r="H101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
@@ -3725,7 +3725,7 @@
           <t>「いいえ」選択</t>
         </is>
       </c>
-      <c r="G102" s="2" t="inlineStr"/>
+      <c r="G102" s="4" t="inlineStr"/>
       <c r="H102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
@@ -3757,7 +3757,7 @@
           <t>国選択+取得経緯表示</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr"/>
+      <c r="G103" s="4" t="inlineStr"/>
       <c r="H103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
@@ -3789,7 +3789,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr"/>
+      <c r="G104" s="4" t="inlineStr"/>
       <c r="H104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
@@ -3821,7 +3821,7 @@
           <t>出生/両親/帰化/その他</t>
         </is>
       </c>
-      <c r="G105" s="2" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr"/>
       <c r="H105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
@@ -3853,7 +3853,7 @@
           <t>「いいえ」選択</t>
         </is>
       </c>
-      <c r="G106" s="2" t="inlineStr"/>
+      <c r="G106" s="4" t="inlineStr"/>
       <c r="H106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
@@ -3885,7 +3885,7 @@
           <t>国選択+取得日+放棄日表示</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr"/>
       <c r="H107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
@@ -3917,7 +3917,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G108" s="2" t="inlineStr"/>
+      <c r="G108" s="4" t="inlineStr"/>
       <c r="H108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
@@ -3949,7 +3949,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G109" s="2" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr"/>
       <c r="H109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
@@ -3981,7 +3981,7 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr"/>
+      <c r="G110" s="4" t="inlineStr"/>
       <c r="H110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
@@ -4013,7 +4013,7 @@
           <t>エラー/警告</t>
         </is>
       </c>
-      <c r="G111" s="2" t="inlineStr"/>
+      <c r="G111" s="4" t="inlineStr"/>
       <c r="H111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
@@ -4045,7 +4045,7 @@
           <t>「いいえ」選択</t>
         </is>
       </c>
-      <c r="G112" s="2" t="inlineStr"/>
+      <c r="G112" s="4" t="inlineStr"/>
       <c r="H112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
@@ -4077,7 +4077,7 @@
           <t>※ご存知でない方は「いいえ」</t>
         </is>
       </c>
-      <c r="G113" s="2" t="inlineStr"/>
+      <c r="G113" s="4" t="inlineStr"/>
       <c r="H113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
@@ -4109,7 +4109,7 @@
           <t>PASS ID入力欄表示</t>
         </is>
       </c>
-      <c r="G114" s="2" t="inlineStr"/>
+      <c r="G114" s="4" t="inlineStr"/>
       <c r="H114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
@@ -4141,7 +4141,7 @@
           <t>エラーなし</t>
         </is>
       </c>
-      <c r="G115" s="2" t="inlineStr"/>
+      <c r="G115" s="4" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
@@ -4173,7 +4173,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G116" s="2" t="inlineStr"/>
+      <c r="G116" s="4" t="inlineStr"/>
       <c r="H116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
@@ -4205,7 +4205,7 @@
           <t>エラー表示</t>
         </is>
       </c>
-      <c r="G117" s="2" t="inlineStr"/>
+      <c r="G117" s="4" t="inlineStr"/>
       <c r="H117" s="4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>